<commit_message>
update SD and fort criteria table
</commit_message>
<xml_diff>
--- a/inst/extdata/fort_peck_tribe_criteria_crosswalk.xlsx
+++ b/inst/extdata/fort_peck_tribe_criteria_crosswalk.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tetratechinc-my.sharepoint.com/personal/k_salkgundersen_tetratech_com/Documents/EPA/R8_AssessmentTool/5_Work/Crosswalks/individual_criteria_crosswalks/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kwong01\TADACommunityHub\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD7FB050-DD07-47CF-9963-5BDED1BFAA5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8812648A-A7E5-40A8-8E4A-550808961698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A9D2C00B-42FB-4D75-83D9-FF6DA97293BD}"/>
+    <workbookView xWindow="28690" yWindow="-110" windowWidth="20710" windowHeight="11020" xr2:uid="{A9D2C00B-42FB-4D75-83D9-FF6DA97293BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AQ$50</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="133">
   <si>
     <t>TADA.ComparableDataIdentifier</t>
   </si>
@@ -472,12 +475,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -492,7 +501,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -507,6 +516,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -843,10 +855,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48473D4D-2A67-413E-80AF-8677973F00EA}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AQ50"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.08984375" customWidth="1"/>
+    <col min="18" max="18" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="4" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:43" s="4" customFormat="1" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -977,7 +998,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5"/>
       <c r="B2" s="5" t="s">
         <v>43</v>
@@ -1046,7 +1067,7 @@
       <c r="AL2" s="5"/>
       <c r="AM2" s="5"/>
     </row>
-    <row r="3" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5"/>
       <c r="B3" s="5" t="s">
         <v>43</v>
@@ -1115,7 +1136,7 @@
       <c r="AL3" s="5"/>
       <c r="AM3" s="5"/>
     </row>
-    <row r="4" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5"/>
       <c r="B4" s="5" t="s">
         <v>43</v>
@@ -1182,7 +1203,7 @@
       <c r="AL4" s="5"/>
       <c r="AM4" s="5"/>
     </row>
-    <row r="5" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5"/>
       <c r="B5" s="5" t="s">
         <v>43</v>
@@ -1249,7 +1270,7 @@
       <c r="AL5" s="5"/>
       <c r="AM5" s="5"/>
     </row>
-    <row r="6" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5"/>
       <c r="B6" s="5" t="s">
         <v>43</v>
@@ -1316,7 +1337,7 @@
       <c r="AL6" s="5"/>
       <c r="AM6" s="5"/>
     </row>
-    <row r="7" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5"/>
       <c r="B7" s="5" t="s">
         <v>43</v>
@@ -1383,7 +1404,7 @@
       <c r="AL7" s="5"/>
       <c r="AM7" s="5"/>
     </row>
-    <row r="8" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5"/>
       <c r="B8" s="5" t="s">
         <v>43</v>
@@ -1450,7 +1471,7 @@
       <c r="AL8" s="5"/>
       <c r="AM8" s="5"/>
     </row>
-    <row r="9" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5"/>
       <c r="B9" s="5" t="s">
         <v>43</v>
@@ -1517,7 +1538,7 @@
       <c r="AL9" s="5"/>
       <c r="AM9" s="5"/>
     </row>
-    <row r="10" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5"/>
       <c r="B10" s="5" t="s">
         <v>43</v>
@@ -1584,7 +1605,7 @@
       <c r="AL10" s="5"/>
       <c r="AM10" s="5"/>
     </row>
-    <row r="11" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5"/>
       <c r="B11" s="5" t="s">
         <v>43</v>
@@ -1651,7 +1672,7 @@
       <c r="AL11" s="5"/>
       <c r="AM11" s="5"/>
     </row>
-    <row r="12" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5"/>
       <c r="B12" s="5" t="s">
         <v>43</v>
@@ -1716,7 +1737,7 @@
       <c r="AL12" s="5"/>
       <c r="AM12" s="5"/>
     </row>
-    <row r="13" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5"/>
       <c r="B13" s="5" t="s">
         <v>43</v>
@@ -1781,7 +1802,7 @@
       <c r="AL13" s="5"/>
       <c r="AM13" s="5"/>
     </row>
-    <row r="14" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5"/>
       <c r="B14" s="5" t="s">
         <v>43</v>
@@ -1846,7 +1867,7 @@
       <c r="AL14" s="5"/>
       <c r="AM14" s="5"/>
     </row>
-    <row r="15" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5"/>
       <c r="B15" s="5" t="s">
         <v>43</v>
@@ -1911,7 +1932,7 @@
       <c r="AL15" s="5"/>
       <c r="AM15" s="5"/>
     </row>
-    <row r="16" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5"/>
       <c r="B16" s="5" t="s">
         <v>43</v>
@@ -1976,7 +1997,7 @@
       <c r="AL16" s="5"/>
       <c r="AM16" s="5"/>
     </row>
-    <row r="17" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5"/>
       <c r="B17" s="5" t="s">
         <v>43</v>
@@ -2041,7 +2062,7 @@
       <c r="AL17" s="5"/>
       <c r="AM17" s="5"/>
     </row>
-    <row r="18" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5"/>
       <c r="B18" s="5" t="s">
         <v>43</v>
@@ -2106,7 +2127,7 @@
       <c r="AL18" s="5"/>
       <c r="AM18" s="5"/>
     </row>
-    <row r="19" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5"/>
       <c r="B19" s="5" t="s">
         <v>43</v>
@@ -2171,7 +2192,7 @@
       <c r="AL19" s="5"/>
       <c r="AM19" s="5"/>
     </row>
-    <row r="20" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5" t="s">
         <v>43</v>
@@ -2236,7 +2257,7 @@
       <c r="AL20" s="5"/>
       <c r="AM20" s="5"/>
     </row>
-    <row r="21" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5"/>
       <c r="B21" s="5" t="s">
         <v>43</v>
@@ -2301,7 +2322,7 @@
       <c r="AL21" s="5"/>
       <c r="AM21" s="5"/>
     </row>
-    <row r="22" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5"/>
       <c r="B22" s="5" t="s">
         <v>43</v>
@@ -2366,7 +2387,7 @@
       <c r="AL22" s="5"/>
       <c r="AM22" s="5"/>
     </row>
-    <row r="23" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5"/>
       <c r="B23" s="5" t="s">
         <v>43</v>
@@ -2431,7 +2452,7 @@
       <c r="AL23" s="5"/>
       <c r="AM23" s="5"/>
     </row>
-    <row r="24" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5"/>
       <c r="B24" s="5" t="s">
         <v>43</v>
@@ -2498,7 +2519,7 @@
       <c r="AL24" s="5"/>
       <c r="AM24" s="5"/>
     </row>
-    <row r="25" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="5"/>
       <c r="B25" s="5" t="s">
         <v>43</v>
@@ -2554,8 +2575,12 @@
       <c r="Y25" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="Z25" s="5"/>
-      <c r="AA25" s="5"/>
+      <c r="Z25" s="6">
+        <v>45809</v>
+      </c>
+      <c r="AA25" s="6">
+        <v>45930</v>
+      </c>
       <c r="AB25" s="5"/>
       <c r="AC25" s="5"/>
       <c r="AD25" s="5"/>
@@ -2569,7 +2594,7 @@
       <c r="AL25" s="5"/>
       <c r="AM25" s="5"/>
     </row>
-    <row r="26" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A26" s="5"/>
       <c r="B26" s="5" t="s">
         <v>43</v>
@@ -2625,8 +2650,12 @@
       <c r="Y26" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="Z26" s="5"/>
-      <c r="AA26" s="5"/>
+      <c r="Z26" s="6">
+        <v>45809</v>
+      </c>
+      <c r="AA26" s="6">
+        <v>45930</v>
+      </c>
       <c r="AB26" s="5"/>
       <c r="AC26" s="5"/>
       <c r="AD26" s="5"/>
@@ -2640,7 +2669,7 @@
       <c r="AL26" s="5"/>
       <c r="AM26" s="5"/>
     </row>
-    <row r="27" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A27" s="5"/>
       <c r="B27" s="5" t="s">
         <v>43</v>
@@ -2694,8 +2723,12 @@
       <c r="Y27" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="Z27" s="5"/>
-      <c r="AA27" s="5"/>
+      <c r="Z27" s="6">
+        <v>45809</v>
+      </c>
+      <c r="AA27" s="6">
+        <v>45930</v>
+      </c>
       <c r="AB27" s="5"/>
       <c r="AC27" s="5"/>
       <c r="AD27" s="5"/>
@@ -2709,7 +2742,7 @@
       <c r="AL27" s="5"/>
       <c r="AM27" s="5"/>
     </row>
-    <row r="28" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A28" s="5"/>
       <c r="B28" s="5" t="s">
         <v>43</v>
@@ -2763,8 +2796,12 @@
       <c r="Y28" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="Z28" s="5"/>
-      <c r="AA28" s="5"/>
+      <c r="Z28" s="6">
+        <v>45809</v>
+      </c>
+      <c r="AA28" s="6">
+        <v>45930</v>
+      </c>
       <c r="AB28" s="5"/>
       <c r="AC28" s="5"/>
       <c r="AD28" s="5"/>
@@ -2778,7 +2815,7 @@
       <c r="AL28" s="5"/>
       <c r="AM28" s="5"/>
     </row>
-    <row r="29" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A29" s="5"/>
       <c r="B29" s="5" t="s">
         <v>43</v>
@@ -2829,9 +2866,15 @@
       <c r="V29" s="5"/>
       <c r="W29" s="5"/>
       <c r="X29" s="5"/>
-      <c r="Y29" s="5"/>
-      <c r="Z29" s="5"/>
-      <c r="AA29" s="5"/>
+      <c r="Y29" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="Z29" s="6">
+        <v>45809</v>
+      </c>
+      <c r="AA29" s="6">
+        <v>45930</v>
+      </c>
       <c r="AB29" s="5"/>
       <c r="AC29" s="5"/>
       <c r="AD29" s="5"/>
@@ -2845,7 +2888,7 @@
       <c r="AL29" s="5"/>
       <c r="AM29" s="5"/>
     </row>
-    <row r="30" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5"/>
       <c r="B30" s="5" t="s">
         <v>43</v>
@@ -2916,7 +2959,7 @@
       <c r="AL30" s="5"/>
       <c r="AM30" s="5"/>
     </row>
-    <row r="31" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="5"/>
       <c r="B31" s="5" t="s">
         <v>43</v>
@@ -2987,7 +3030,7 @@
       <c r="AL31" s="5"/>
       <c r="AM31" s="5"/>
     </row>
-    <row r="32" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5"/>
       <c r="B32" s="5" t="s">
         <v>43</v>
@@ -3058,7 +3101,7 @@
       <c r="AL32" s="5"/>
       <c r="AM32" s="5"/>
     </row>
-    <row r="33" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5"/>
       <c r="B33" s="5" t="s">
         <v>43</v>
@@ -3129,7 +3172,7 @@
       <c r="AL33" s="5"/>
       <c r="AM33" s="5"/>
     </row>
-    <row r="34" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5"/>
       <c r="B34" s="5" t="s">
         <v>43</v>
@@ -3200,7 +3243,7 @@
       <c r="AL34" s="5"/>
       <c r="AM34" s="5"/>
     </row>
-    <row r="35" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5"/>
       <c r="B35" s="5" t="s">
         <v>43</v>
@@ -3271,7 +3314,7 @@
       <c r="AL35" s="5"/>
       <c r="AM35" s="5"/>
     </row>
-    <row r="36" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5"/>
       <c r="B36" s="5" t="s">
         <v>43</v>
@@ -3342,7 +3385,7 @@
       <c r="AL36" s="5"/>
       <c r="AM36" s="5"/>
     </row>
-    <row r="37" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5"/>
       <c r="B37" s="5" t="s">
         <v>43</v>
@@ -3413,7 +3456,7 @@
       <c r="AL37" s="5"/>
       <c r="AM37" s="5"/>
     </row>
-    <row r="38" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5"/>
       <c r="B38" s="5" t="s">
         <v>43</v>
@@ -3484,7 +3527,7 @@
       <c r="AL38" s="5"/>
       <c r="AM38" s="5"/>
     </row>
-    <row r="39" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="5"/>
       <c r="B39" s="5" t="s">
         <v>43</v>
@@ -3555,7 +3598,7 @@
       <c r="AL39" s="5"/>
       <c r="AM39" s="5"/>
     </row>
-    <row r="40" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5"/>
       <c r="B40" s="5" t="s">
         <v>43</v>
@@ -3636,7 +3679,7 @@
       </c>
       <c r="AM40" s="5"/>
     </row>
-    <row r="41" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="5"/>
       <c r="B41" s="5" t="s">
         <v>43</v>
@@ -3717,7 +3760,7 @@
       </c>
       <c r="AM41" s="5"/>
     </row>
-    <row r="42" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5"/>
       <c r="B42" s="5" t="s">
         <v>43</v>
@@ -3798,7 +3841,7 @@
       </c>
       <c r="AM42" s="5"/>
     </row>
-    <row r="43" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="5"/>
       <c r="B43" s="5" t="s">
         <v>43</v>
@@ -3879,7 +3922,7 @@
       </c>
       <c r="AM43" s="5"/>
     </row>
-    <row r="44" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="5"/>
       <c r="B44" s="5" t="s">
         <v>43</v>
@@ -3960,7 +4003,7 @@
       </c>
       <c r="AM44" s="5"/>
     </row>
-    <row r="45" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="5"/>
       <c r="B45" s="5" t="s">
         <v>43</v>
@@ -4041,7 +4084,7 @@
       </c>
       <c r="AM45" s="5"/>
     </row>
-    <row r="46" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="5"/>
       <c r="B46" s="5" t="s">
         <v>43</v>
@@ -4122,7 +4165,7 @@
       </c>
       <c r="AM46" s="5"/>
     </row>
-    <row r="47" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="5"/>
       <c r="B47" s="5" t="s">
         <v>43</v>
@@ -4203,7 +4246,7 @@
       </c>
       <c r="AM47" s="5"/>
     </row>
-    <row r="48" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="5"/>
       <c r="B48" s="5" t="s">
         <v>43</v>
@@ -4284,7 +4327,7 @@
       </c>
       <c r="AM48" s="5"/>
     </row>
-    <row r="49" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="5"/>
       <c r="B49" s="5" t="s">
         <v>43</v>
@@ -4365,7 +4408,7 @@
       </c>
       <c r="AM49" s="5"/>
     </row>
-    <row r="50" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="5"/>
       <c r="B50" s="5" t="s">
         <v>43</v>
@@ -4447,6 +4490,13 @@
       <c r="AM50" s="5"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AQ50" xr:uid="{48473D4D-2A67-413E-80AF-8677973F00EA}">
+    <filterColumn colId="17">
+      <filters>
+        <filter val="n-season"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>